<commit_message>
QAQC'd July 2024 SMARTX Dionex Data
</commit_message>
<xml_diff>
--- a/SMARTX/Porewater/Sulfate_Chloride/2024/Raw Data/SMARTX and LTREB 2024 Dionex Run Dates.xlsx
+++ b/SMARTX/Porewater/Sulfate_Chloride/2024/Raw Data/SMARTX and LTREB 2024 Dionex Run Dates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/GCREW/SMARTX/Porewater/Sulfate_Chloride/2024/Raw Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{1898BD2C-5046-4422-A88F-4B03B9BA45C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{302646F8-D6B8-4F3F-BD18-2A82372EF19F}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{1898BD2C-5046-4422-A88F-4B03B9BA45C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A36E8DA9-0B57-414F-BE14-501BBBC788DD}"/>
   <bookViews>
-    <workbookView xWindow="6915" yWindow="645" windowWidth="14025" windowHeight="12945" xr2:uid="{B4279EF9-9A73-4C24-89F6-1FBD8C43B9DF}"/>
+    <workbookView xWindow="-19320" yWindow="690" windowWidth="19440" windowHeight="14880" xr2:uid="{B4279EF9-9A73-4C24-89F6-1FBD8C43B9DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -128,6 +128,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -450,7 +454,7 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>